<commit_message>
Update unit counts for Nativa/Gestion and Servidores in La Libertad addressing scheme script
</commit_message>
<xml_diff>
--- a/LA-LIBERTAD-ESQUEMA-DIRECCIONAMIENTO-IA.xlsx
+++ b/LA-LIBERTAD-ESQUEMA-DIRECCIONAMIENTO-IA.xlsx
@@ -607,10 +607,10 @@
         </is>
       </c>
       <c r="B14" s="6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C14" s="6">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
@@ -621,19 +621,19 @@
         <v>99</v>
       </c>
       <c r="F14" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14" s="6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>/28</t>
+          <t>/29</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>255.255.255.240</t>
+          <t>255.255.255.248</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
@@ -648,12 +648,12 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>10.192.45.46</t>
+          <t>10.192.45.38</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>10.192.45.47</t>
+          <t>10.192.45.39</t>
         </is>
       </c>
     </row>
@@ -664,10 +664,10 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C15" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
@@ -695,22 +695,22 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>10.192.45.48</t>
+          <t>10.192.45.40</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>10.192.45.49</t>
+          <t>10.192.45.41</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>10.192.45.54</t>
+          <t>10.192.45.46</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>10.192.45.55</t>
+          <t>10.192.45.47</t>
         </is>
       </c>
     </row>
@@ -721,13 +721,13 @@
         </is>
       </c>
       <c r="B16" s="1">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C16" s="1">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="G16" s="1">
-        <v>294</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18">

</xml_diff>